<commit_message>
feat: 配置改为 channels×models 分离，新增 --sample 示例模式与 --models/--channels 过滤
</commit_message>
<xml_diff>
--- a/report_template.xlsx
+++ b/report_template.xlsx
@@ -580,7 +580,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -4191,7 +4191,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>模型@渠道</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">

</xml_diff>